<commit_message>
Added TIVERS for context
</commit_message>
<xml_diff>
--- a/rules/CORE-000146/negative/01/data/unit-test-coreid-CG0256-negative 1.xlsx
+++ b/rules/CORE-000146/negative/01/data/unit-test-coreid-CG0256-negative 1.xlsx
@@ -1,43 +1,140 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr codeName="ThisWorkbook"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Repos\Verisian\core-contributor\rules\CORE-000146\negative\01\data\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{65C96574-DC2B-4CEA-9547-64B1E635C295}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <bookViews>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
     <sheet name="Library" sheetId="1" r:id="rId1"/>
     <sheet name="Datasets" sheetId="2" r:id="rId2"/>
     <sheet name="Validation" sheetId="3" r:id="rId3"/>
     <sheet name="ti.xpt" sheetId="4" r:id="rId4"/>
   </sheets>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
-<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
-  <metadataTypes count="1">
-    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
-  </metadataTypes>
-  <futureMetadata name="XLDAPR" count="1">
-    <bk>
-      <extLst>
-        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
-          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
-        </ext>
-      </extLst>
-    </bk>
-  </futureMetadata>
-  <cellMetadata count="1">
-    <bk>
-      <rc t="1" v="0"/>
-    </bk>
-  </cellMetadata>
-</metadata>
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="33">
+  <si>
+    <t>Product</t>
+  </si>
+  <si>
+    <t>Version</t>
+  </si>
+  <si>
+    <t>sdtmig</t>
+  </si>
+  <si>
+    <t>3-4</t>
+  </si>
+  <si>
+    <t>Filename</t>
+  </si>
+  <si>
+    <t>Label</t>
+  </si>
+  <si>
+    <t>ti.xpt</t>
+  </si>
+  <si>
+    <t>Trial Inclusion/Exclusion Criteria</t>
+  </si>
+  <si>
+    <t>Error group</t>
+  </si>
+  <si>
+    <t>Sheet</t>
+  </si>
+  <si>
+    <t>Error level</t>
+  </si>
+  <si>
+    <t>Row num</t>
+  </si>
+  <si>
+    <t>Variable</t>
+  </si>
+  <si>
+    <t>Error value</t>
+  </si>
+  <si>
+    <t>Record</t>
+  </si>
+  <si>
+    <t>IETESTCD</t>
+  </si>
+  <si>
+    <t>INCL01</t>
+  </si>
+  <si>
+    <t>STUDYID</t>
+  </si>
+  <si>
+    <t>DOMAIN</t>
+  </si>
+  <si>
+    <t>IETEST</t>
+  </si>
+  <si>
+    <t>IECAT</t>
+  </si>
+  <si>
+    <t>Study Identifier</t>
+  </si>
+  <si>
+    <t>Domain Abbreviation</t>
+  </si>
+  <si>
+    <t>Incl/Excl Criterion Short Name</t>
+  </si>
+  <si>
+    <t>Inclusion/Exclusion Criterion</t>
+  </si>
+  <si>
+    <t>Inclusion/Exclusion Category</t>
+  </si>
+  <si>
+    <t>Char</t>
+  </si>
+  <si>
+    <t>CDISCPILOT01</t>
+  </si>
+  <si>
+    <t>TI</t>
+  </si>
+  <si>
+    <t>Males and postmenopausal females at least 50 years of age.</t>
+  </si>
+  <si>
+    <t>INCLUSION</t>
+  </si>
+  <si>
+    <t>TIVERS</t>
+  </si>
+  <si>
+    <t>[ABSENT]</t>
+  </si>
+</sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" mc:Ignorable="x14ac">
-  <numFmts count="0"/>
-  <fonts count="7" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <name val="Calibri"/>
     </font>
@@ -46,23 +143,14 @@
       <name val="Calibri"/>
     </font>
     <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <b/>
-    </font>
-    <font>
+      <i/>
       <sz val="11"/>
       <name val="Calibri"/>
     </font>
     <font>
+      <i/>
       <sz val="11"/>
       <name val="Calibri"/>
-      <i/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <i/>
     </font>
     <font>
       <sz val="11"/>
@@ -71,42 +159,28 @@
   </fonts>
   <fills count="5">
     <fill>
-      <patternFill patternType="none">
-        <bgColor/>
-      </patternFill>
+      <patternFill patternType="none"/>
     </fill>
     <fill>
-      <patternFill patternType="gray125">
-        <bgColor/>
+      <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFCC"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFFCC"/>
-        <bgColor/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFCC"/>
-        <bgColor/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFF00"/>
-        <bgColor/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -115,24 +189,32 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs>
+  <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="1" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
-  <cellStyles>
+  <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium4"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -457,239 +539,287 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B2"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="3" t="str">
-        <v>Product</v>
-      </c>
-      <c r="B1" s="3" t="str">
-        <v>Version</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="4" t="str">
-        <v>sdtmig</v>
-      </c>
-      <c r="B2" s="4" t="str">
-        <v>3-4</v>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>3</v>
       </c>
     </row>
   </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B2"/>
+    <ignoredError sqref="A1:B2" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:B2"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="3" t="str">
-        <v>Filename</v>
-      </c>
-      <c r="B1" s="3" t="str">
-        <v>Label</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="4" t="str">
-        <v>ti.xpt</v>
-      </c>
-      <c r="B2" s="4" t="str">
-        <v>Trial Inclusion/Exclusion Criteria</v>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>7</v>
       </c>
     </row>
   </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B2"/>
+    <ignoredError sqref="A1:B2" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+  <dimension ref="A1:F5"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="3" t="str">
-        <v>Error group</v>
-      </c>
-      <c r="B1" s="3" t="str">
-        <v>Sheet</v>
-      </c>
-      <c r="C1" s="3" t="str">
-        <v>Error level</v>
-      </c>
-      <c r="D1" s="3" t="str">
-        <v>Row num</v>
-      </c>
-      <c r="E1" s="3" t="str">
-        <v>Variable</v>
-      </c>
-      <c r="F1" s="3" t="str">
-        <v>Error value</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="4">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" s="3">
         <v>1</v>
       </c>
-      <c r="B2" s="4" t="str">
-        <v>ti.xpt</v>
-      </c>
-      <c r="C2" s="4" t="str">
-        <v>Record</v>
-      </c>
-      <c r="D2" s="4">
+      <c r="B2" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="D2" s="3">
         <v>5</v>
       </c>
-      <c r="E2" s="4" t="str">
-        <v>IETESTCD</v>
-      </c>
-      <c r="F2" s="4" t="str">
-        <v>INCL01</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="4">
+      <c r="E2" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="F2" s="3" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="3">
+        <v>1</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="D3" s="3">
+        <v>5</v>
+      </c>
+      <c r="E3" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="F3" s="7" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" s="3">
         <v>2</v>
       </c>
-      <c r="B3" s="4" t="str">
-        <v>ti.xpt</v>
-      </c>
-      <c r="C3" s="4" t="str">
-        <v>Record</v>
-      </c>
-      <c r="D3" s="4">
+      <c r="B4" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="E3" s="4" t="str">
-        <v>IETESTCD</v>
-      </c>
-      <c r="F3" s="4" t="str">
-        <v>INCL01</v>
+      <c r="C4" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="D4" s="3">
+        <v>6</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="F4" s="3" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" s="3">
+        <v>2</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="D5" s="3">
+        <v>6</v>
+      </c>
+      <c r="E5" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="F5" s="7" t="s">
+        <v>32</v>
       </c>
     </row>
   </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F3"/>
+    <ignoredError sqref="A4:F4 A1:F2" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:E6"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="3" t="str">
-        <v>STUDYID</v>
-      </c>
-      <c r="B1" s="3" t="str">
-        <v>DOMAIN</v>
-      </c>
-      <c r="C1" s="3" t="str">
-        <v>IETESTCD</v>
-      </c>
-      <c r="D1" s="3" t="str">
-        <v>IETEST</v>
-      </c>
-      <c r="E1" s="3" t="str">
-        <v>IECAT</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="5" t="str">
-        <v>Study Identifier</v>
-      </c>
-      <c r="B2" s="6" t="str">
-        <v>Domain Abbreviation</v>
-      </c>
-      <c r="C2" s="6" t="str">
-        <v>Incl/Excl Criterion Short Name</v>
-      </c>
-      <c r="D2" s="6" t="str">
-        <v>Inclusion/Exclusion Criterion</v>
-      </c>
-      <c r="E2" s="6" t="str">
-        <v>Inclusion/Exclusion Category</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="6" t="str">
-        <v>Char</v>
-      </c>
-      <c r="B3" s="6" t="str">
-        <v>Char</v>
-      </c>
-      <c r="C3" s="6" t="str">
-        <v>Char</v>
-      </c>
-      <c r="D3" s="6" t="str">
-        <v>Char</v>
-      </c>
-      <c r="E3" s="6" t="str">
-        <v>Char</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="6">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="B2" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="C2" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="D2" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="E2" s="5" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A3" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="B3" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="D3" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="E3" s="5" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4" s="5">
         <v>12</v>
       </c>
-      <c r="B4" s="6">
+      <c r="B4" s="5">
         <v>2</v>
       </c>
-      <c r="C4" s="6">
+      <c r="C4" s="5">
         <v>7</v>
       </c>
-      <c r="D4" s="6">
+      <c r="D4" s="5">
         <v>196</v>
       </c>
-      <c r="E4" s="6">
+      <c r="E4" s="5">
         <v>9</v>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="4" t="str">
-        <v>CDISCPILOT01</v>
-      </c>
-      <c r="B5" s="4" t="str">
-        <v>TI</v>
-      </c>
-      <c r="C5" s="7" t="str">
-        <v>INCL01</v>
-      </c>
-      <c r="D5" s="4" t="str">
-        <v>Males and postmenopausal females at least 50 years of age.</v>
-      </c>
-      <c r="E5" s="4" t="str">
-        <v>INCLUSION</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="4" t="str">
-        <v>CDISCPILOT01</v>
-      </c>
-      <c r="B6" s="4" t="str">
-        <v>TI</v>
-      </c>
-      <c r="C6" s="7" t="str">
-        <v>INCL01</v>
-      </c>
-      <c r="D6" s="4" t="str">
-        <v>Males and postmenopausal females at least 50 years of age.</v>
-      </c>
-      <c r="E6" s="4" t="str">
-        <v>INCLUSION</v>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A5" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="C5" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A6" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="C6" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="D6" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="E6" s="3" t="s">
+        <v>30</v>
       </c>
     </row>
   </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E6"/>
+    <ignoredError sqref="A1:E6" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>